<commit_message>
ELEC study rev 2: disclosed Q1-26 P&L lines + FY25 facilities (10.9bn) replace derived anchors; full rebuild & re-reconciliation
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDB3U7m8U6NX4ju3RCn348
</commit_message>
<xml_diff>
--- a/engine/elec_study/ELEC_Valuation_Model_05082026_public.xlsx
+++ b/engine/elec_study/ELEC_Valuation_Model_05082026_public.xlsx
@@ -76,7 +76,7 @@
     <t xml:space="preserve">year, closes to the reported net profit within 0.8% using the derived lines.</t>
   </si>
   <si>
-    <t xml:space="preserve">Discount convention. Each explicit year is discounted at its own forward WACC, gliding 22.6% -&gt; 14.1% on the</t>
+    <t xml:space="preserve">Discount convention. Each explicit year is discounted at its own forward WACC, gliding 21.4% -&gt; 13.9% on the</t>
   </si>
   <si>
     <t xml:space="preserve">same easing calendar as the interest forecast; the terminal value is capitalised at the terminal WACC and</t>
@@ -211,7 +211,7 @@
     <t xml:space="preserve">Kd pre-tax (marginal EGP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Corridor + levered margin; effective-rate checks 23.4% (FY24) / 23.2% (FY25) inside 150bp</t>
+    <t xml:space="preserve">Corridor + credit margin; effective-rate checks 23.5% (FY24) / 21.7% (FY25, disclosed debt path) inside 150bp</t>
   </si>
   <si>
     <t xml:space="preserve">Kd after tax</t>
@@ -220,10 +220,10 @@
     <t xml:space="preserve">Market cap (spot × shares)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total debt for weights (FY24 disclosed vintage)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Simply Wall St, 22-May-2025 — the sourced debt print</t>
+    <t xml:space="preserve">Total debt for weights (FY25 disclosed facilities)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY25 results coverage: EGP 10.9bn bank facilities vs 8.96bn FY24 (matches the FY24 debt print — cross-validated)</t>
   </si>
   <si>
     <t xml:space="preserve">Equity weight E/(D+E)</t>
@@ -268,7 +268,7 @@
     <t xml:space="preserve">Net debt (FY25, derived)</t>
   </si>
   <si>
-    <t xml:space="preserve">Derived from twice-sourced FY25 assets 16,460 + FY24 anchors; FY24-vintage sourced alt: 8,172</t>
+    <t xml:space="preserve">Disclosed facilities 10,900 less estimated cash ~700; FY24-vintage sourced alt: 8,172 — worth ±EGP 0.6/sh, see Sensitivity</t>
   </si>
   <si>
     <t xml:space="preserve">Non-controlling interests</t>
@@ -346,7 +346,7 @@
     <t xml:space="preserve">EBITDA margin</t>
   </si>
   <si>
-    <t xml:space="preserve">Between the 1Q26 trough (~14%) and windfall prints (~25%)</t>
+    <t xml:space="preserve">1Q26 DISCLOSED: gross margin 5.7%, operating ~0 — the trough; windfall prints ~25% the ceiling</t>
   </si>
   <si>
     <t xml:space="preserve">D&amp;A (% of revenue)</t>
@@ -361,7 +361,7 @@
     <t xml:space="preserve">Net working capital (% of revenue)</t>
   </si>
   <si>
-    <t xml:space="preserve">From ~111% FY25e; NOT full reversion to FY24 76%</t>
+    <t xml:space="preserve">From ~117% FY25e; NOT full reversion to FY24 76%</t>
   </si>
   <si>
     <t xml:space="preserve">Forward Kd path</t>
@@ -391,7 +391,7 @@
     <t xml:space="preserve">Net working capital FY25 (derived)</t>
   </si>
   <si>
-    <t xml:space="preserve">~111% of FY25 revenue — construction in study §1.6</t>
+    <t xml:space="preserve">~117% of FY25 revenue — construction in study §1.6</t>
   </si>
   <si>
     <t xml:space="preserve">EV → equity bridge</t>
@@ -406,7 +406,7 @@
     <t xml:space="preserve">+ Surplus / non-core assets</t>
   </si>
   <si>
-    <t xml:space="preserve">− Net debt (FY25, derived; ±1,000 sensitized)</t>
+    <t xml:space="preserve">− Net debt (FY25: disclosed facilities − est. cash)</t>
   </si>
   <si>
     <t xml:space="preserve">− Non-controlling interests</t>
@@ -1734,23 +1734,23 @@
       </c>
       <c r="C6" s="17" t="n">
         <f aca="false">Assumptions!B52</f>
-        <v>12000</v>
+        <v>12640</v>
       </c>
       <c r="D6" s="24" t="n">
         <f aca="false">DCF!B13</f>
-        <v>9394.35408</v>
+        <v>9742.29312</v>
       </c>
       <c r="E6" s="24" t="n">
         <f aca="false">DCF!C13</f>
-        <v>10213.7505192</v>
+        <v>10511.2383984</v>
       </c>
       <c r="F6" s="24" t="n">
         <f aca="false">DCF!D13</f>
-        <v>10884.089873664</v>
+        <v>11106.2141568</v>
       </c>
       <c r="G6" s="24" t="n">
         <f aca="false">DCF!E13</f>
-        <v>11361.6570824064</v>
+        <v>11483.8254381312</v>
       </c>
       <c r="H6" s="24" t="n">
         <f aca="false">DCF!F13</f>
@@ -1829,23 +1829,23 @@
       </c>
       <c r="C9" s="30" t="n">
         <f aca="false">SUM(C6:C8)</f>
-        <v>15660</v>
+        <v>16300</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">SUM(D6:D8)</f>
-        <v>13080.449508</v>
+        <v>13428.388548</v>
       </c>
       <c r="E9" s="19" t="n">
         <f aca="false">SUM(E6:E8)</f>
-        <v>13929.59473512</v>
+        <v>14227.08261432</v>
       </c>
       <c r="F9" s="19" t="n">
         <f aca="false">SUM(F6:F8)</f>
-        <v>14633.2527320544</v>
+        <v>14855.3770151904</v>
       </c>
       <c r="G9" s="19" t="n">
         <f aca="false">SUM(G6:G8)</f>
-        <v>15147.4704475142</v>
+        <v>15269.638803239</v>
       </c>
       <c r="H9" s="19" t="n">
         <f aca="false">SUM(H6:H8)</f>
@@ -1857,31 +1857,31 @@
         <v>195</v>
       </c>
       <c r="B11" s="17" t="n">
-        <v>8172</v>
+        <v>8172.4</v>
       </c>
       <c r="C11" s="17" t="n">
         <f aca="false">Assumptions!B28</f>
-        <v>8800</v>
+        <v>10200</v>
       </c>
       <c r="D11" s="24" t="n">
         <f aca="false">Assumptions!$B$28-'Cash Flow'!C12</f>
-        <v>7270.727816</v>
+        <v>9033.083036</v>
       </c>
       <c r="E11" s="24" t="n">
         <f aca="false">D11-'Cash Flow'!D12</f>
-        <v>8189.0352764</v>
+        <v>10379.02835424</v>
       </c>
       <c r="F11" s="24" t="n">
         <f aca="false">E11-'Cash Flow'!E12</f>
-        <v>8649.4032824488</v>
+        <v>11294.8295195952</v>
       </c>
       <c r="G11" s="24" t="n">
         <f aca="false">F11-'Cash Flow'!F12</f>
-        <v>8532.72383745838</v>
+        <v>11627.4953041941</v>
       </c>
       <c r="H11" s="24" t="n">
         <f aca="false">G11-'Cash Flow'!G12</f>
-        <v>7981.42929540173</v>
+        <v>11392.9662497003</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1898,23 +1898,23 @@
       </c>
       <c r="D12" s="24" t="n">
         <f aca="false">C12+'Income Statement'!E14</f>
-        <v>3049.721692</v>
+        <v>2395.305512</v>
       </c>
       <c r="E12" s="24" t="n">
         <f aca="false">D12+'Income Statement'!F14</f>
-        <v>2980.55945872</v>
+        <v>1848.05426008</v>
       </c>
       <c r="F12" s="24" t="n">
         <f aca="false">E12+'Income Statement'!G14</f>
-        <v>3223.8494496056</v>
+        <v>1560.5474955952</v>
       </c>
       <c r="G12" s="24" t="n">
         <f aca="false">F12+'Income Statement'!H14</f>
-        <v>3854.74661005587</v>
+        <v>1642.14349904497</v>
       </c>
       <c r="H12" s="24" t="n">
         <f aca="false">G12+'Income Statement'!I14</f>
-        <v>4694.84714504595</v>
+        <v>2043.31019074738</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1923,31 +1923,31 @@
       </c>
       <c r="B13" s="31" t="n">
         <f aca="false">B9-B11-B12</f>
-        <v>2378.31</v>
+        <v>2377.91</v>
       </c>
       <c r="C13" s="31" t="n">
         <f aca="false">C9-C11-C12</f>
-        <v>2760</v>
+        <v>2000</v>
       </c>
       <c r="D13" s="31" t="n">
         <f aca="false">$C13</f>
-        <v>2760</v>
+        <v>2000</v>
       </c>
       <c r="E13" s="31" t="n">
         <f aca="false">$C13</f>
-        <v>2760</v>
+        <v>2000</v>
       </c>
       <c r="F13" s="31" t="n">
         <f aca="false">$C13</f>
-        <v>2760</v>
+        <v>2000</v>
       </c>
       <c r="G13" s="31" t="n">
         <f aca="false">$C13</f>
-        <v>2760</v>
+        <v>2000</v>
       </c>
       <c r="H13" s="31" t="n">
         <f aca="false">$C13</f>
-        <v>2760</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1960,23 +1960,23 @@
       </c>
       <c r="C14" s="30" t="n">
         <f aca="false">C11+C12+C13</f>
-        <v>15660</v>
+        <v>16300</v>
       </c>
       <c r="D14" s="19" t="n">
         <f aca="false">D11+D12+D13</f>
-        <v>13080.449508</v>
+        <v>13428.388548</v>
       </c>
       <c r="E14" s="19" t="n">
         <f aca="false">E11+E12+E13</f>
-        <v>13929.59473512</v>
+        <v>14227.08261432</v>
       </c>
       <c r="F14" s="19" t="n">
         <f aca="false">F11+F12+F13</f>
-        <v>14633.2527320544</v>
+        <v>14855.3770151904</v>
       </c>
       <c r="G14" s="19" t="n">
         <f aca="false">G11+G12+G13</f>
-        <v>15147.4704475142</v>
+        <v>15269.638803239</v>
       </c>
       <c r="H14" s="19" t="n">
         <f aca="false">H11+H12+H13</f>
@@ -2086,23 +2086,23 @@
       </c>
       <c r="C6" s="24" t="n">
         <f aca="false">'Income Statement'!E14</f>
-        <v>-1050.278308</v>
+        <v>-1704.694488</v>
       </c>
       <c r="D6" s="24" t="n">
         <f aca="false">'Income Statement'!F14</f>
-        <v>-69.1622332799998</v>
+        <v>-547.25125192</v>
       </c>
       <c r="E6" s="24" t="n">
         <f aca="false">'Income Statement'!G14</f>
-        <v>243.2899908856</v>
+        <v>-287.5067644848</v>
       </c>
       <c r="F6" s="24" t="n">
         <f aca="false">'Income Statement'!H14</f>
-        <v>630.897160450264</v>
+        <v>81.5960034497662</v>
       </c>
       <c r="G6" s="24" t="n">
         <f aca="false">'Income Statement'!I14</f>
-        <v>840.100534990083</v>
+        <v>401.166691702412</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2136,23 +2136,23 @@
       </c>
       <c r="C8" s="24" t="n">
         <f aca="false">DCF!B14</f>
-        <v>2605.64592</v>
+        <v>2897.70688</v>
       </c>
       <c r="D8" s="24" t="n">
         <f aca="false">DCF!C14</f>
-        <v>-819.3964392</v>
+        <v>-768.945278399999</v>
       </c>
       <c r="E8" s="24" t="n">
         <f aca="false">DCF!D14</f>
-        <v>-670.339354464002</v>
+        <v>-594.975758400002</v>
       </c>
       <c r="F8" s="24" t="n">
         <f aca="false">DCF!E14</f>
-        <v>-477.567208742401</v>
+        <v>-377.611281331201</v>
       </c>
       <c r="G8" s="24" t="n">
         <f aca="false">DCF!F14</f>
-        <v>-249.223445678594</v>
+        <v>-127.055089953794</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2186,23 +2186,23 @@
       </c>
       <c r="C10" s="19" t="n">
         <f aca="false">SUM(C6:C9)</f>
-        <v>1529.272184</v>
+        <v>1166.916964</v>
       </c>
       <c r="D10" s="19" t="n">
         <f aca="false">SUM(D6:D9)</f>
-        <v>-918.3074604</v>
+        <v>-1345.94531824</v>
       </c>
       <c r="E10" s="19" t="n">
         <f aca="false">SUM(E6:E9)</f>
-        <v>-460.368006048802</v>
+        <v>-915.801165355201</v>
       </c>
       <c r="F10" s="19" t="n">
         <f aca="false">SUM(F6:F9)</f>
-        <v>116.679444990423</v>
+        <v>-332.665784598875</v>
       </c>
       <c r="G10" s="19" t="n">
         <f aca="false">SUM(G6:G9)</f>
-        <v>551.294542056654</v>
+        <v>234.529054493782</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2231,23 +2231,23 @@
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">C10+C11</f>
-        <v>1529.272184</v>
+        <v>1166.916964</v>
       </c>
       <c r="D12" s="19" t="n">
         <f aca="false">D10+D11</f>
-        <v>-918.3074604</v>
+        <v>-1345.94531824</v>
       </c>
       <c r="E12" s="19" t="n">
         <f aca="false">E10+E11</f>
-        <v>-460.368006048802</v>
+        <v>-915.801165355201</v>
       </c>
       <c r="F12" s="19" t="n">
         <f aca="false">F10+F11</f>
-        <v>116.679444990423</v>
+        <v>-332.665784598875</v>
       </c>
       <c r="G12" s="19" t="n">
         <f aca="false">G10+G11</f>
-        <v>551.294542056654</v>
+        <v>234.529054493782</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2256,23 +2256,23 @@
       </c>
       <c r="C14" s="24" t="n">
         <f aca="false">DCF!B15</f>
-        <v>3368.2848033</v>
+        <v>3289.5732238</v>
       </c>
       <c r="D14" s="24" t="n">
         <f aca="false">DCF!C15</f>
-        <v>280.564994142</v>
+        <v>177.314084022002</v>
       </c>
       <c r="E14" s="24" t="n">
         <f aca="false">DCF!D15</f>
-        <v>690.727190451838</v>
+        <v>636.981046943039</v>
       </c>
       <c r="F14" s="24" t="n">
         <f aca="false">DCF!E15</f>
-        <v>1114.28646635174</v>
+        <v>1119.56191807622</v>
       </c>
       <c r="G14" s="24" t="n">
         <f aca="false">DCF!F15</f>
-        <v>1521.10598029391</v>
+        <v>1541.01942227705</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2281,23 +2281,23 @@
       </c>
       <c r="C15" s="24" t="n">
         <f aca="false">'Balance Sheet'!D11</f>
-        <v>7270.727816</v>
+        <v>9033.083036</v>
       </c>
       <c r="D15" s="24" t="n">
         <f aca="false">'Balance Sheet'!E11</f>
-        <v>8189.0352764</v>
+        <v>10379.02835424</v>
       </c>
       <c r="E15" s="24" t="n">
         <f aca="false">'Balance Sheet'!F11</f>
-        <v>8649.4032824488</v>
+        <v>11294.8295195952</v>
       </c>
       <c r="F15" s="24" t="n">
         <f aca="false">'Balance Sheet'!G11</f>
-        <v>8532.72383745838</v>
+        <v>11627.4953041941</v>
       </c>
       <c r="G15" s="24" t="n">
         <f aca="false">'Balance Sheet'!H11</f>
-        <v>7981.42929540173</v>
+        <v>11392.9662497003</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2423,23 +2423,23 @@
       </c>
       <c r="E7" s="24" t="n">
         <f aca="false">'Income Statement'!E7</f>
-        <v>1130.80188</v>
+        <v>652.3857</v>
       </c>
       <c r="F7" s="24" t="n">
         <f aca="false">'Income Statement'!F7</f>
-        <v>1586.6020224</v>
+        <v>1388.2767696</v>
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">'Income Statement'!G7</f>
-        <v>1943.58747744</v>
+        <v>1776.994265088</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">'Income Statement'!H7</f>
-        <v>2260.1145809088</v>
+        <v>2137.946225184</v>
       </c>
       <c r="I7" s="24" t="n">
         <f aca="false">'Income Statement'!I7</f>
-        <v>2506.8946594729</v>
+        <v>2374.95283529011</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2457,23 +2457,23 @@
       </c>
       <c r="E8" s="24" t="n">
         <f aca="false">'Income Statement'!E9</f>
-        <v>1017.721692</v>
+        <v>539.305512</v>
       </c>
       <c r="F8" s="24" t="n">
         <f aca="false">'Income Statement'!F9</f>
-        <v>1457.69060808</v>
+        <v>1259.36535528</v>
       </c>
       <c r="G8" s="24" t="n">
         <f aca="false">'Income Statement'!G9</f>
-        <v>1799.2066934016</v>
+        <v>1632.6134810496</v>
       </c>
       <c r="H8" s="24" t="n">
         <f aca="false">'Income Statement'!H9</f>
-        <v>2101.29571846656</v>
+        <v>1979.12736274176</v>
       </c>
       <c r="I8" s="24" t="n">
         <f aca="false">'Income Statement'!I9</f>
-        <v>2335.37028803528</v>
+        <v>2203.42846385249</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2491,23 +2491,23 @@
       </c>
       <c r="E9" s="24" t="n">
         <f aca="false">'Income Statement'!E14</f>
-        <v>-1050.278308</v>
+        <v>-1704.694488</v>
       </c>
       <c r="F9" s="24" t="n">
         <f aca="false">'Income Statement'!F14</f>
-        <v>-69.1622332799998</v>
+        <v>-547.25125192</v>
       </c>
       <c r="G9" s="24" t="n">
         <f aca="false">'Income Statement'!G14</f>
-        <v>243.2899908856</v>
+        <v>-287.5067644848</v>
       </c>
       <c r="H9" s="24" t="n">
         <f aca="false">'Income Statement'!H14</f>
-        <v>630.897160450264</v>
+        <v>81.5960034497662</v>
       </c>
       <c r="I9" s="24" t="n">
         <f aca="false">'Income Statement'!I14</f>
-        <v>840.100534990083</v>
+        <v>401.166691702412</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2516,27 +2516,27 @@
       </c>
       <c r="D10" s="24" t="n">
         <f aca="false">Assumptions!B28</f>
-        <v>8800</v>
+        <v>10200</v>
       </c>
       <c r="E10" s="24" t="n">
         <f aca="false">'Balance Sheet'!D11</f>
-        <v>7270.727816</v>
+        <v>9033.083036</v>
       </c>
       <c r="F10" s="24" t="n">
         <f aca="false">'Balance Sheet'!E11</f>
-        <v>8189.0352764</v>
+        <v>10379.02835424</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">'Balance Sheet'!F11</f>
-        <v>8649.4032824488</v>
+        <v>11294.8295195952</v>
       </c>
       <c r="H10" s="24" t="n">
         <f aca="false">'Balance Sheet'!G11</f>
-        <v>8532.72383745838</v>
+        <v>11627.4953041941</v>
       </c>
       <c r="I10" s="24" t="n">
         <f aca="false">'Balance Sheet'!H11</f>
-        <v>7981.42929540173</v>
+        <v>11392.9662497003</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2549,23 +2549,23 @@
       </c>
       <c r="E11" s="24" t="n">
         <f aca="false">'Balance Sheet'!D12</f>
-        <v>3049.721692</v>
+        <v>2395.305512</v>
       </c>
       <c r="F11" s="24" t="n">
         <f aca="false">'Balance Sheet'!E12</f>
-        <v>2980.55945872</v>
+        <v>1848.05426008</v>
       </c>
       <c r="G11" s="24" t="n">
         <f aca="false">'Balance Sheet'!F12</f>
-        <v>3223.8494496056</v>
+        <v>1560.5474955952</v>
       </c>
       <c r="H11" s="24" t="n">
         <f aca="false">'Balance Sheet'!G12</f>
-        <v>3854.74661005587</v>
+        <v>1642.14349904497</v>
       </c>
       <c r="I11" s="24" t="n">
         <f aca="false">'Balance Sheet'!H12</f>
-        <v>4694.84714504595</v>
+        <v>2043.31019074738</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2574,23 +2574,23 @@
       </c>
       <c r="E12" s="24" t="n">
         <f aca="false">DCF!B15</f>
-        <v>3368.2848033</v>
+        <v>3289.5732238</v>
       </c>
       <c r="F12" s="24" t="n">
         <f aca="false">DCF!C15</f>
-        <v>280.564994142</v>
+        <v>177.314084022002</v>
       </c>
       <c r="G12" s="24" t="n">
         <f aca="false">DCF!D15</f>
-        <v>690.727190451838</v>
+        <v>636.981046943039</v>
       </c>
       <c r="H12" s="24" t="n">
         <f aca="false">DCF!E15</f>
-        <v>1114.28646635174</v>
+        <v>1119.56191807622</v>
       </c>
       <c r="I12" s="24" t="n">
         <f aca="false">DCF!F15</f>
-        <v>1521.10598029391</v>
+        <v>1541.01942227705</v>
       </c>
     </row>
   </sheetData>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">DCF!B31</f>
-        <v>0.533988597838447</v>
+        <v>0.0233762361074855</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2983,102 +2983,102 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="n">
-        <v>0.121349976678297</v>
+        <v>0.118723393761621</v>
       </c>
       <c r="B9" s="29" t="n">
-        <v>0.98</v>
+        <v>0.49</v>
       </c>
       <c r="C9" s="29" t="n">
-        <v>1.07</v>
+        <v>0.57</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>1.17</v>
+        <v>0.66</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>1.3</v>
+        <v>0.77</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>1.48</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="n">
-        <v>0.131349976678297</v>
+        <v>0.128723393761621</v>
       </c>
       <c r="B10" s="29" t="n">
-        <v>0.71</v>
+        <v>0.21</v>
       </c>
       <c r="C10" s="29" t="n">
-        <v>0.76</v>
+        <v>0.25</v>
       </c>
       <c r="D10" s="29" t="n">
-        <v>0.81</v>
+        <v>0.3</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.88</v>
+        <v>0.35</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.97</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="n">
-        <v>0.141349976678297</v>
+        <v>0.138723393761621</v>
       </c>
       <c r="B11" s="29" t="n">
-        <v>0.48</v>
+        <v>-0.01</v>
       </c>
       <c r="C11" s="29" t="n">
-        <v>0.51</v>
+        <v>0.01</v>
       </c>
       <c r="D11" s="29" t="n">
-        <v>0.53</v>
+        <v>0.02</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.57</v>
+        <v>0.04</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="n">
-        <v>0.151349976678297</v>
+        <v>0.148723393761621</v>
       </c>
       <c r="B12" s="29" t="n">
-        <v>0.29</v>
+        <v>-0.2</v>
       </c>
       <c r="C12" s="29" t="n">
-        <v>0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="D12" s="29" t="n">
-        <v>0.31</v>
+        <v>-0.2</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.32</v>
+        <v>-0.2</v>
       </c>
       <c r="F12" s="29" t="n">
-        <v>0.32</v>
+        <v>-0.21</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="n">
-        <v>0.161349976678297</v>
+        <v>0.158723393761621</v>
       </c>
       <c r="B13" s="29" t="n">
-        <v>0.13</v>
+        <v>-0.36</v>
       </c>
       <c r="C13" s="29" t="n">
-        <v>0.13</v>
+        <v>-0.37</v>
       </c>
       <c r="D13" s="29" t="n">
-        <v>0.13</v>
+        <v>-0.38</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.12</v>
+        <v>-0.4</v>
       </c>
       <c r="F13" s="29" t="n">
-        <v>0.11</v>
+        <v>-0.42</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3091,119 +3091,119 @@
         <v>255</v>
       </c>
       <c r="B16" s="34" t="n">
-        <v>0.121349976678297</v>
+        <v>0.118723393761621</v>
       </c>
       <c r="C16" s="34" t="n">
-        <v>0.131349976678297</v>
+        <v>0.128723393761621</v>
       </c>
       <c r="D16" s="34" t="n">
-        <v>0.141349976678297</v>
+        <v>0.138723393761621</v>
       </c>
       <c r="E16" s="34" t="n">
-        <v>0.151349976678297</v>
+        <v>0.148723393761621</v>
       </c>
       <c r="F16" s="34" t="n">
-        <v>0.161349976678297</v>
+        <v>0.158723393761621</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="n">
-        <v>0.205730752476676</v>
+        <v>0.194188789049045</v>
       </c>
       <c r="B17" s="29" t="n">
-        <v>1.3</v>
+        <v>0.79</v>
       </c>
       <c r="C17" s="29" t="n">
-        <v>0.93</v>
+        <v>0.42</v>
       </c>
       <c r="D17" s="29" t="n">
-        <v>0.64</v>
+        <v>0.13</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.41</v>
+        <v>-0.1</v>
       </c>
       <c r="F17" s="29" t="n">
-        <v>0.21</v>
+        <v>-0.29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="n">
-        <v>0.215730752476676</v>
+        <v>0.204188789049045</v>
       </c>
       <c r="B18" s="29" t="n">
-        <v>1.23</v>
+        <v>0.72</v>
       </c>
       <c r="C18" s="29" t="n">
-        <v>0.87</v>
+        <v>0.36</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>0.59</v>
+        <v>0.08</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.36</v>
+        <v>-0.15</v>
       </c>
       <c r="F18" s="29" t="n">
-        <v>0.17</v>
+        <v>-0.33</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="n">
-        <v>0.225730752476676</v>
+        <v>0.214188789049045</v>
       </c>
       <c r="B19" s="29" t="n">
-        <v>1.17</v>
+        <v>0.66</v>
       </c>
       <c r="C19" s="29" t="n">
-        <v>0.81</v>
+        <v>0.3</v>
       </c>
       <c r="D19" s="29" t="n">
-        <v>0.53</v>
+        <v>0.02</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.31</v>
+        <v>-0.2</v>
       </c>
       <c r="F19" s="29" t="n">
-        <v>0.13</v>
+        <v>-0.38</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="n">
-        <v>0.235730752476676</v>
+        <v>0.224188789049045</v>
       </c>
       <c r="B20" s="29" t="n">
-        <v>1.11</v>
+        <v>0.59</v>
       </c>
       <c r="C20" s="29" t="n">
-        <v>0.76</v>
+        <v>0.24</v>
       </c>
       <c r="D20" s="29" t="n">
-        <v>0.48</v>
+        <v>-0.03</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.26</v>
+        <v>-0.24</v>
       </c>
       <c r="F20" s="29" t="n">
-        <v>0.08</v>
+        <v>-0.42</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="n">
-        <v>0.245730752476676</v>
+        <v>0.234188789049045</v>
       </c>
       <c r="B21" s="29" t="n">
-        <v>1.04</v>
+        <v>0.53</v>
       </c>
       <c r="C21" s="29" t="n">
-        <v>0.7</v>
+        <v>0.19</v>
       </c>
       <c r="D21" s="29" t="n">
-        <v>0.43</v>
+        <v>-0.08</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0.22</v>
+        <v>-0.29</v>
       </c>
       <c r="F21" s="29" t="n">
-        <v>0.04</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3236,19 +3236,19 @@
         <v>-0.03</v>
       </c>
       <c r="B25" s="29" t="n">
-        <v>-0.53</v>
+        <v>-1.08</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>-0.34</v>
+        <v>-0.89</v>
       </c>
       <c r="D25" s="29" t="n">
-        <v>-0.16</v>
+        <v>-0.7</v>
       </c>
       <c r="E25" s="29" t="n">
-        <v>0.03</v>
+        <v>-0.5</v>
       </c>
       <c r="F25" s="29" t="n">
-        <v>0.22</v>
+        <v>-0.31</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3256,19 +3256,19 @@
         <v>-0.015</v>
       </c>
       <c r="B26" s="29" t="n">
-        <v>-0.19</v>
+        <v>-0.72</v>
       </c>
       <c r="C26" s="29" t="n">
-        <v>0</v>
+        <v>-0.53</v>
       </c>
       <c r="D26" s="29" t="n">
-        <v>0.19</v>
+        <v>-0.34</v>
       </c>
       <c r="E26" s="29" t="n">
-        <v>0.38</v>
+        <v>-0.14</v>
       </c>
       <c r="F26" s="29" t="n">
-        <v>0.56</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3276,19 +3276,19 @@
         <v>0</v>
       </c>
       <c r="B27" s="29" t="n">
-        <v>0.16</v>
+        <v>-0.36</v>
       </c>
       <c r="C27" s="29" t="n">
-        <v>0.35</v>
+        <v>-0.17</v>
       </c>
       <c r="D27" s="29" t="n">
-        <v>0.53</v>
+        <v>0.02</v>
       </c>
       <c r="E27" s="29" t="n">
-        <v>0.72</v>
+        <v>0.22</v>
       </c>
       <c r="F27" s="29" t="n">
-        <v>0.91</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3296,19 +3296,19 @@
         <v>0.015</v>
       </c>
       <c r="B28" s="29" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C28" s="29" t="n">
-        <v>0.69</v>
+        <v>0.19</v>
       </c>
       <c r="D28" s="29" t="n">
-        <v>0.88</v>
+        <v>0.38</v>
       </c>
       <c r="E28" s="29" t="n">
-        <v>1.07</v>
+        <v>0.58</v>
       </c>
       <c r="F28" s="29" t="n">
-        <v>1.25</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3316,19 +3316,19 @@
         <v>0.03</v>
       </c>
       <c r="B29" s="29" t="n">
-        <v>0.85</v>
+        <v>0.36</v>
       </c>
       <c r="C29" s="29" t="n">
-        <v>1.04</v>
+        <v>0.55</v>
       </c>
       <c r="D29" s="29" t="n">
-        <v>1.22</v>
+        <v>0.74</v>
       </c>
       <c r="E29" s="29" t="n">
-        <v>1.41</v>
+        <v>0.94</v>
       </c>
       <c r="F29" s="29" t="n">
-        <v>1.6</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3361,13 +3361,13 @@
         <v>0.24556</v>
       </c>
       <c r="C33" s="12" t="n">
-        <v>0.210441148329856</v>
+        <v>0.200499163004575</v>
       </c>
       <c r="D33" s="12" t="n">
-        <v>0.129976201011162</v>
+        <v>0.128539824971898</v>
       </c>
       <c r="E33" s="29" t="n">
-        <v>0.86</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3378,13 +3378,13 @@
         <v>0.262498</v>
       </c>
       <c r="C34" s="12" t="n">
-        <v>0.218001941589273</v>
+        <v>0.207268758301291</v>
       </c>
       <c r="D34" s="12" t="n">
-        <v>0.135600595571833</v>
+        <v>0.133575655692091</v>
       </c>
       <c r="E34" s="29" t="n">
-        <v>0.69</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3395,13 +3395,13 @@
         <v>0.26438</v>
       </c>
       <c r="C35" s="12" t="n">
-        <v>0.218842029729208</v>
+        <v>0.208020935556482</v>
       </c>
       <c r="D35" s="12" t="n">
-        <v>0.136225528300797</v>
+        <v>0.134135192438779</v>
       </c>
       <c r="E35" s="29" t="n">
-        <v>0.67</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3412,13 +3412,13 @@
         <v>0.2798124</v>
       </c>
       <c r="C36" s="12" t="n">
-        <v>0.225730752476676</v>
+        <v>0.214188789049045</v>
       </c>
       <c r="D36" s="12" t="n">
-        <v>0.141349976678297</v>
+        <v>0.138723393761621</v>
       </c>
       <c r="E36" s="29" t="n">
-        <v>0.53</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3429,13 +3429,13 @@
         <v>0.2832</v>
       </c>
       <c r="C37" s="12" t="n">
-        <v>0.22724291112856</v>
+        <v>0.215542708108388</v>
       </c>
       <c r="D37" s="12" t="n">
-        <v>0.142474855590432</v>
+        <v>0.13973055990566</v>
       </c>
       <c r="E37" s="29" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3446,13 +3446,13 @@
         <v>0.297315</v>
       </c>
       <c r="C38" s="12" t="n">
-        <v>0.233543572178074</v>
+        <v>0.221184037522318</v>
       </c>
       <c r="D38" s="12" t="n">
-        <v>0.147161851057658</v>
+        <v>0.14392708550582</v>
       </c>
       <c r="E38" s="29" t="n">
-        <v>0.4</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3463,13 +3463,13 @@
         <v>0.31143</v>
       </c>
       <c r="C39" s="12" t="n">
-        <v>0.239844233227587</v>
+        <v>0.226825366936248</v>
       </c>
       <c r="D39" s="12" t="n">
-        <v>0.151848846524884</v>
+        <v>0.14812361110598</v>
       </c>
       <c r="E39" s="29" t="n">
-        <v>0.3</v>
+        <v>-0.19</v>
       </c>
     </row>
   </sheetData>
@@ -3559,23 +3559,23 @@
       </c>
       <c r="E6" s="29" t="n">
         <f aca="false">'Income Statement'!E14/Assumptions!$B$6</f>
-        <v>-0.316965598656371</v>
+        <v>-0.514463171141811</v>
       </c>
       <c r="F6" s="29" t="n">
         <f aca="false">'Income Statement'!F14/Assumptions!$B$6</f>
-        <v>-0.0208726092017952</v>
+        <v>-0.165156053742159</v>
       </c>
       <c r="G6" s="29" t="n">
         <f aca="false">'Income Statement'!G14/Assumptions!$B$6</f>
-        <v>0.0734229746732591</v>
+        <v>-0.0867672435282562</v>
       </c>
       <c r="H6" s="29" t="n">
         <f aca="false">'Income Statement'!H14/Assumptions!$B$6</f>
-        <v>0.190399720368901</v>
+        <v>0.0246250216579951</v>
       </c>
       <c r="I6" s="29" t="n">
         <f aca="false">'Income Statement'!I14/Assumptions!$B$6</f>
-        <v>0.2535356266776</v>
+        <v>0.121068901097832</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3602,17 +3602,17 @@
         <f aca="false">IF('Income Statement'!F14&gt;0,Assumptions!$B$5/('Income Statement'!F14/Assumptions!$B$6),"n.m.")</f>
         <v>n.m.</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="26" t="str">
         <f aca="false">IF('Income Statement'!G14&gt;0,Assumptions!$B$5/('Income Statement'!G14/Assumptions!$B$6),"n.m.")</f>
-        <v>29.8271761631255</v>
+        <v>n.m.</v>
       </c>
       <c r="H7" s="26" t="n">
         <f aca="false">IF('Income Statement'!H14&gt;0,Assumptions!$B$5/('Income Statement'!H14/Assumptions!$B$6),"n.m.")</f>
-        <v>11.5021177329297</v>
+        <v>88.9339319337802</v>
       </c>
       <c r="I7" s="26" t="n">
         <f aca="false">IF('Income Statement'!I14&gt;0,Assumptions!$B$5/('Income Statement'!I14/Assumptions!$B$6),"n.m.")</f>
-        <v>8.63783929974008</v>
+        <v>18.0888731965141</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3633,23 +3633,23 @@
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">'Income Statement'!E7/'Income Statement'!E6</f>
-        <v>0.13</v>
+        <v>0.075</v>
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">'Income Statement'!F7/'Income Statement'!F6</f>
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="G8" s="12" t="n">
         <f aca="false">'Income Statement'!G7/'Income Statement'!G6</f>
-        <v>0.175</v>
+        <v>0.16</v>
       </c>
       <c r="H8" s="12" t="n">
         <f aca="false">'Income Statement'!H7/'Income Statement'!H6</f>
-        <v>0.185</v>
+        <v>0.175</v>
       </c>
       <c r="I8" s="12" t="n">
         <f aca="false">'Income Statement'!I7/'Income Statement'!I6</f>
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3670,23 +3670,23 @@
       </c>
       <c r="E9" s="12" t="n">
         <f aca="false">'Income Statement'!E14/'Income Statement'!E6</f>
-        <v>-0.12074279540462</v>
+        <v>-0.195976224800758</v>
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">'Income Statement'!F14/'Income Statement'!F6</f>
-        <v>-0.00697462701330789</v>
+        <v>-0.0551872486427003</v>
       </c>
       <c r="G9" s="12" t="n">
         <f aca="false">'Income Statement'!G14/'Income Statement'!G6</f>
-        <v>0.0219057536124172</v>
+        <v>-0.0258870178825759</v>
       </c>
       <c r="H9" s="12" t="n">
         <f aca="false">'Income Statement'!H14/'Income Statement'!H6</f>
-        <v>0.0516416183804128</v>
+        <v>0.00667898024538954</v>
       </c>
       <c r="I9" s="12" t="n">
         <f aca="false">'Income Statement'!I14/'Income Statement'!I6</f>
-        <v>0.0636720418406721</v>
+        <v>0.0304048162276929</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3732,23 +3732,23 @@
       </c>
       <c r="E11" s="29" t="n">
         <f aca="false">'Balance Sheet'!D12/Assumptions!$B$6</f>
-        <v>0.920381630732586</v>
+        <v>0.722884058247145</v>
       </c>
       <c r="F11" s="29" t="n">
         <f aca="false">'Balance Sheet'!E12/Assumptions!$B$6</f>
-        <v>0.899509021530791</v>
+        <v>0.557728004504987</v>
       </c>
       <c r="G11" s="29" t="n">
         <f aca="false">'Balance Sheet'!F12/Assumptions!$B$6</f>
-        <v>0.97293199620405</v>
+        <v>0.470960760976731</v>
       </c>
       <c r="H11" s="29" t="n">
         <f aca="false">'Balance Sheet'!G12/Assumptions!$B$6</f>
-        <v>1.16333171657295</v>
+        <v>0.495585782634726</v>
       </c>
       <c r="I11" s="29" t="n">
         <f aca="false">'Balance Sheet'!H12/Assumptions!$B$6</f>
-        <v>1.41686734325055</v>
+        <v>0.616654683732558</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3763,23 +3763,23 @@
       </c>
       <c r="E12" s="26" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!D12/Assumptions!$B$6)</f>
-        <v>2.37944774957846</v>
+        <v>3.02953146499084</v>
       </c>
       <c r="F12" s="26" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!E12/Assumptions!$B$6)</f>
-        <v>2.43466151820584</v>
+        <v>3.92664521471132</v>
       </c>
       <c r="G12" s="26" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!F12/Assumptions!$B$6)</f>
-        <v>2.25092813119973</v>
+        <v>4.65006892603565</v>
       </c>
       <c r="H12" s="26" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!G12/Assumptions!$B$6)</f>
-        <v>1.88252410623816</v>
+        <v>4.41901296755753</v>
       </c>
       <c r="I12" s="26" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!H12/Assumptions!$B$6)</f>
-        <v>1.5456634034459</v>
+        <v>3.55142036178841</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3790,27 +3790,27 @@
       <c r="C13" s="36"/>
       <c r="D13" s="26" t="n">
         <f aca="false">Assumptions!$B$28/'Income Statement'!D7</f>
-        <v>3.06481994188459</v>
+        <v>3.55240493263895</v>
       </c>
       <c r="E13" s="26" t="n">
         <f aca="false">'Balance Sheet'!D11/'Income Statement'!E7</f>
-        <v>6.42970969945681</v>
+        <v>13.8462308968452</v>
       </c>
       <c r="F13" s="26" t="n">
         <f aca="false">'Balance Sheet'!E11/'Income Statement'!F7</f>
-        <v>5.16136697217411</v>
+        <v>7.47619536789518</v>
       </c>
       <c r="G13" s="26" t="n">
         <f aca="false">'Balance Sheet'!F11/'Income Statement'!G7</f>
-        <v>4.45022587500995</v>
+        <v>6.35614292150564</v>
       </c>
       <c r="H13" s="26" t="n">
         <f aca="false">'Balance Sheet'!G11/'Income Statement'!H7</f>
-        <v>3.77535011257143</v>
+        <v>5.43862851517389</v>
       </c>
       <c r="I13" s="26" t="n">
         <f aca="false">'Balance Sheet'!H11/'Income Statement'!I7</f>
-        <v>3.18379125554478</v>
+        <v>4.79713368636585</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3819,27 +3819,27 @@
       </c>
       <c r="D14" s="12" t="n">
         <f aca="false">Assumptions!$B$28/Assumptions!$B$34</f>
-        <v>2.14634146341463</v>
+        <v>2.48780487804878</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">'Balance Sheet'!D11/'Balance Sheet'!D12</f>
-        <v>2.38406272778021</v>
+        <v>3.77116112777517</v>
       </c>
       <c r="F14" s="12" t="n">
         <f aca="false">'Balance Sheet'!E11/'Balance Sheet'!E12</f>
-        <v>2.7474826084888</v>
+        <v>5.61619243462619</v>
       </c>
       <c r="G14" s="12" t="n">
         <f aca="false">'Balance Sheet'!F11/'Balance Sheet'!F12</f>
-        <v>2.68294268006434</v>
+        <v>7.2377351868341</v>
       </c>
       <c r="H14" s="12" t="n">
         <f aca="false">'Balance Sheet'!G11/'Balance Sheet'!G12</f>
-        <v>2.21356283580329</v>
+        <v>7.08068162797975</v>
       </c>
       <c r="I14" s="12" t="n">
         <f aca="false">'Balance Sheet'!H11/'Balance Sheet'!H12</f>
-        <v>1.70004028860105</v>
+        <v>5.57573994457157</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3848,23 +3848,23 @@
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">'Income Statement'!E14/'Balance Sheet'!D12</f>
-        <v>-0.344384968226799</v>
+        <v>-0.711681445001409</v>
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">'Income Statement'!F14/'Balance Sheet'!E12</f>
-        <v>-0.0232044467617168</v>
+        <v>-0.296122935208791</v>
       </c>
       <c r="G15" s="12" t="n">
         <f aca="false">'Income Statement'!G14/'Balance Sheet'!F12</f>
-        <v>0.0754656799855725</v>
+        <v>-0.184234549282426</v>
       </c>
       <c r="H15" s="12" t="n">
         <f aca="false">'Income Statement'!H14/'Balance Sheet'!G12</f>
-        <v>0.163667608865508</v>
+        <v>0.0496887169100755</v>
       </c>
       <c r="I15" s="12" t="n">
         <f aca="false">'Income Statement'!I14/'Balance Sheet'!H12</f>
-        <v>0.178940976997849</v>
+        <v>0.196331762802826</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4081,14 +4081,14 @@
         <v>25</v>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">DCF!B31</f>
-        <v>0.533988597838447</v>
+        <v>0.0233762361074855</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>2.81</v>
+        <v>2.36</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">Assumptions!B35</f>
@@ -4104,10 +4104,10 @@
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">'Relative &amp; Normalized'!C6</f>
-        <v>0.439283407880179</v>
+        <v>0.05</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.92</v>
+        <v>0.05</v>
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">Assumptions!B36</f>
@@ -4119,14 +4119,14 @@
         <v>27</v>
       </c>
       <c r="B8" s="7" t="n">
-        <v>0.75</v>
+        <v>0.55</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">'Relative &amp; Normalized'!C7</f>
-        <v>1.36704346653529</v>
+        <v>1.11377559810627</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>2.26</v>
+        <v>1.92</v>
       </c>
       <c r="E8" s="9" t="n">
         <f aca="false">Assumptions!B37</f>
@@ -4158,15 +4158,15 @@
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">SUMPRODUCT(B6:B9,$E$6:$E$9)</f>
-        <v>0.302</v>
+        <v>0.246</v>
       </c>
       <c r="C10" s="11" t="n">
         <f aca="false">SUMPRODUCT(C6:C9,$E$6:$E$9)</f>
-        <v>0.756704789598169</v>
+        <v>0.423949589643946</v>
       </c>
       <c r="D10" s="11" t="n">
         <f aca="false">SUMPRODUCT(D6:D9,$E$6:$E$9)</f>
-        <v>2.046</v>
+        <v>1.624</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="B13" s="12" t="n">
         <f aca="false">C10/Assumptions!B5-1</f>
-        <v>-0.654472698813621</v>
+        <v>-0.806415712491349</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4251,15 +4251,15 @@
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">Summary!B6</f>
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">Summary!C6</f>
-        <v>0.533988597838447</v>
+        <v>0.0233762361074855</v>
       </c>
       <c r="D6" s="8" t="n">
         <f aca="false">Summary!D6</f>
-        <v>2.81</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4272,11 +4272,11 @@
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">Summary!C7</f>
-        <v>0.439283407880179</v>
+        <v>0.05</v>
       </c>
       <c r="D7" s="8" t="n">
         <f aca="false">Summary!D7</f>
-        <v>0.92</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4285,15 +4285,15 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">Summary!B8</f>
-        <v>0.75</v>
+        <v>0.55</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">Summary!C8</f>
-        <v>1.36704346653529</v>
+        <v>1.11377559810627</v>
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">Summary!D8</f>
-        <v>2.26</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4319,15 +4319,15 @@
       </c>
       <c r="B10" s="15" t="n">
         <f aca="false">Summary!B10</f>
-        <v>0.302</v>
+        <v>0.246</v>
       </c>
       <c r="C10" s="15" t="n">
         <f aca="false">Summary!C10</f>
-        <v>0.756704789598169</v>
+        <v>0.423949589643946</v>
       </c>
       <c r="D10" s="15" t="n">
         <f aca="false">Summary!D10</f>
-        <v>2.046</v>
+        <v>1.624</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4494,7 +4494,7 @@
         <v>57</v>
       </c>
       <c r="B15" s="18" t="n">
-        <v>0.235</v>
+        <v>0.22</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>58</v>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">B15*(1-B7)</f>
-        <v>0.182125</v>
+        <v>0.1705</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4523,7 +4523,7 @@
         <v>61</v>
       </c>
       <c r="B18" s="17" t="n">
-        <v>9000</v>
+        <v>10900</v>
       </c>
       <c r="C18" s="13" t="s">
         <v>62</v>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">B17/(B17+B18)</f>
-        <v>0.446380520688198</v>
+        <v>0.399669104777182</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="B20" s="20" t="n">
         <f aca="false">B19*B14+(1-B19)*B16</f>
-        <v>0.225730752476676</v>
+        <v>0.214188789049045</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="B25" s="20" t="n">
         <f aca="false">B19*B23+(1-B19)*B24*(1-B7)</f>
-        <v>0.141349976678297</v>
+        <v>0.138723393761621</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4619,7 +4619,7 @@
         <v>76</v>
       </c>
       <c r="B28" s="17" t="n">
-        <v>8800</v>
+        <v>10200</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>77</v>
@@ -4770,19 +4770,19 @@
         <v>102</v>
       </c>
       <c r="C42" s="18" t="n">
-        <v>0.13</v>
+        <v>0.075</v>
       </c>
       <c r="D42" s="18" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E42" s="18" t="n">
         <v>0.16</v>
       </c>
-      <c r="E42" s="18" t="n">
+      <c r="F42" s="18" t="n">
         <v>0.175</v>
       </c>
-      <c r="F42" s="18" t="n">
-        <v>0.185</v>
-      </c>
       <c r="G42" s="18" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="H42" s="13" t="s">
         <v>103</v>
@@ -4836,16 +4836,16 @@
         <v>107</v>
       </c>
       <c r="C45" s="18" t="n">
-        <v>1.08</v>
+        <v>1.12</v>
       </c>
       <c r="D45" s="18" t="n">
-        <v>1.03</v>
+        <v>1.06</v>
       </c>
       <c r="E45" s="18" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="F45" s="18" t="n">
-        <v>0.93</v>
+        <v>0.94</v>
       </c>
       <c r="G45" s="18" t="n">
         <v>0.88</v>
@@ -4859,16 +4859,16 @@
         <v>109</v>
       </c>
       <c r="C46" s="18" t="n">
-        <v>0.235</v>
+        <v>0.22</v>
       </c>
       <c r="D46" s="18" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="E46" s="18" t="n">
-        <v>0.19</v>
+        <v>0.185</v>
       </c>
       <c r="F46" s="18" t="n">
-        <v>0.17</v>
+        <v>0.168</v>
       </c>
       <c r="G46" s="18" t="n">
         <v>0.155</v>
@@ -4887,15 +4887,15 @@
       </c>
       <c r="D47" s="12" t="n">
         <f aca="false">($C$46-D46)/($C$46-$G$46)</f>
-        <v>0.3125</v>
+        <v>0.307692307692308</v>
       </c>
       <c r="E47" s="12" t="n">
         <f aca="false">($C$46-E46)/($C$46-$G$46)</f>
-        <v>0.5625</v>
+        <v>0.538461538461539</v>
       </c>
       <c r="F47" s="12" t="n">
         <f aca="false">($C$46-F46)/($C$46-$G$46)</f>
-        <v>0.8125</v>
+        <v>0.8</v>
       </c>
       <c r="G47" s="12" t="n">
         <f aca="false">($C$46-G46)/($C$46-$G$46)</f>
@@ -4908,23 +4908,23 @@
       </c>
       <c r="C48" s="12" t="n">
         <f aca="false">$B$20-($B$20-$B$25)*C47</f>
-        <v>0.225730752476676</v>
+        <v>0.214188789049045</v>
       </c>
       <c r="D48" s="12" t="n">
         <f aca="false">$B$20-($B$20-$B$25)*D47</f>
-        <v>0.199361760039683</v>
+        <v>0.190968667422146</v>
       </c>
       <c r="E48" s="12" t="n">
         <f aca="false">$B$20-($B$20-$B$25)*E47</f>
-        <v>0.178266566090088</v>
+        <v>0.173553576201971</v>
       </c>
       <c r="F48" s="12" t="n">
         <f aca="false">$B$20-($B$20-$B$25)*F47</f>
-        <v>0.157171372140493</v>
+        <v>0.153816472819106</v>
       </c>
       <c r="G48" s="12" t="n">
         <f aca="false">$B$20-($B$20-$B$25)*G47</f>
-        <v>0.141349976678297</v>
+        <v>0.138723393761621</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4933,23 +4933,23 @@
       </c>
       <c r="C49" s="22" t="n">
         <f aca="false">1/(1+C48)</f>
-        <v>0.815839855514295</v>
+        <v>0.82359515177471</v>
       </c>
       <c r="D49" s="22" t="n">
         <f aca="false">C49/(1+D48)</f>
-        <v>0.6802283370176</v>
+        <v>0.691533853327463</v>
       </c>
       <c r="E49" s="22" t="n">
         <f aca="false">D49/(1+E48)</f>
-        <v>0.577312771654756</v>
+        <v>0.589264834048317</v>
       </c>
       <c r="F49" s="22" t="n">
         <f aca="false">E49/(1+F48)</f>
-        <v>0.498899977612532</v>
+        <v>0.510709326768904</v>
       </c>
       <c r="G49" s="22" t="n">
         <f aca="false">F49/(1+G48)</f>
-        <v>0.437113933330507</v>
+        <v>0.448492873305996</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4973,7 +4973,7 @@
         <v>117</v>
       </c>
       <c r="B52" s="17" t="n">
-        <v>12000</v>
+        <v>12640</v>
       </c>
       <c r="C52" s="13" t="s">
         <v>118</v>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="B5" s="23" t="n">
         <f aca="false">DCF!B26</f>
-        <v>10569.3927776594</v>
+        <v>10277.4581021109</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="B7" s="24" t="n">
         <f aca="false">-Assumptions!B28</f>
-        <v>-8800</v>
+        <v>-10200</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="B9" s="23" t="n">
         <f aca="false">B5+B6+B7+B8</f>
-        <v>1769.39277765935</v>
+        <v>77.4581021109334</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5068,7 +5068,7 @@
       </c>
       <c r="B10" s="15" t="n">
         <f aca="false">B9/Assumptions!B6</f>
-        <v>0.533988597838447</v>
+        <v>0.0233762361074855</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="B11" s="25" t="n">
         <f aca="false">B10/Assumptions!B5-1</f>
-        <v>-0.756169590028107</v>
+        <v>-0.989325919585623</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5100,7 +5100,7 @@
       </c>
       <c r="B15" s="6" t="n">
         <f aca="false">B14+Assumptions!B28</f>
-        <v>16056.65341687</v>
+        <v>17456.65341687</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5109,7 +5109,7 @@
       </c>
       <c r="B16" s="26" t="n">
         <f aca="false">B15/Segments!F9</f>
-        <v>10.1201518655457</v>
+        <v>12.5743322939126</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5118,7 +5118,7 @@
       </c>
       <c r="B17" s="26" t="n">
         <f aca="false">B15/Segments!D9</f>
-        <v>5.59213086272187</v>
+        <v>6.07971585347624</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5294,23 +5294,23 @@
       </c>
       <c r="E9" s="24" t="n">
         <f aca="false">E6*Assumptions!C42</f>
-        <v>1130.80188</v>
+        <v>652.3857</v>
       </c>
       <c r="F9" s="24" t="n">
         <f aca="false">F6*Assumptions!D42</f>
-        <v>1586.6020224</v>
+        <v>1388.2767696</v>
       </c>
       <c r="G9" s="24" t="n">
         <f aca="false">G6*Assumptions!E42</f>
-        <v>1943.58747744</v>
+        <v>1776.994265088</v>
       </c>
       <c r="H9" s="24" t="n">
         <f aca="false">H6*Assumptions!F42</f>
-        <v>2260.1145809088</v>
+        <v>2137.946225184</v>
       </c>
       <c r="I9" s="24" t="n">
         <f aca="false">I6*Assumptions!G42</f>
-        <v>2506.8946594729</v>
+        <v>2374.95283529011</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5331,23 +5331,23 @@
       </c>
       <c r="E10" s="12" t="n">
         <f aca="false">E9/E6</f>
-        <v>0.13</v>
+        <v>0.075</v>
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">F9/F6</f>
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="G10" s="12" t="n">
         <f aca="false">G9/G6</f>
-        <v>0.175</v>
+        <v>0.16</v>
       </c>
       <c r="H10" s="12" t="n">
         <f aca="false">H9/H6</f>
-        <v>0.185</v>
+        <v>0.175</v>
       </c>
       <c r="I10" s="12" t="n">
         <f aca="false">I9/I6</f>
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5399,23 +5399,23 @@
       </c>
       <c r="E12" s="19" t="n">
         <f aca="false">E9-E11</f>
-        <v>1017.721692</v>
+        <v>539.305512</v>
       </c>
       <c r="F12" s="19" t="n">
         <f aca="false">F9-F11</f>
-        <v>1457.69060808</v>
+        <v>1259.36535528</v>
       </c>
       <c r="G12" s="19" t="n">
         <f aca="false">G9-G11</f>
-        <v>1799.2066934016</v>
+        <v>1632.6134810496</v>
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">H9-H11</f>
-        <v>2101.29571846656</v>
+        <v>1979.12736274176</v>
       </c>
       <c r="I12" s="19" t="n">
         <f aca="false">I9-I11</f>
-        <v>2335.37028803528</v>
+        <v>2203.42846385249</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5483,7 +5483,7 @@
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">MAX((Assumptions!B31*Segments!F9-'Balance Sheet'!D11)/Assumptions!B6,0.05)</f>
-        <v>0.439283407880179</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">(Segments!G12-Assumptions!B24*6000)*(1-Assumptions!B7)*Assumptions!B32/Assumptions!B6</f>
-        <v>1.36704346653529</v>
+        <v>1.11377559810627</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5504,7 +5504,7 @@
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">(Segments!G12-Assumptions!B24*6000)*(1-Assumptions!B7)/Assumptions!B6</f>
-        <v>0.210314379466968</v>
+        <v>0.17135009201635</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5616,23 +5616,23 @@
       </c>
       <c r="B7" s="24" t="n">
         <f aca="false">Segments!E9</f>
-        <v>1130.80188</v>
+        <v>652.3857</v>
       </c>
       <c r="C7" s="24" t="n">
         <f aca="false">Segments!F9</f>
-        <v>1586.6020224</v>
+        <v>1388.2767696</v>
       </c>
       <c r="D7" s="24" t="n">
         <f aca="false">Segments!G9</f>
-        <v>1943.58747744</v>
+        <v>1776.994265088</v>
       </c>
       <c r="E7" s="24" t="n">
         <f aca="false">Segments!H9</f>
-        <v>2260.1145809088</v>
+        <v>2137.946225184</v>
       </c>
       <c r="F7" s="24" t="n">
         <f aca="false">Segments!I9</f>
-        <v>2506.8946594729</v>
+        <v>2374.95283529011</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5666,23 +5666,23 @@
       </c>
       <c r="B9" s="24" t="n">
         <f aca="false">Segments!E12</f>
-        <v>1017.721692</v>
+        <v>539.305512</v>
       </c>
       <c r="C9" s="24" t="n">
         <f aca="false">Segments!F12</f>
-        <v>1457.69060808</v>
+        <v>1259.36535528</v>
       </c>
       <c r="D9" s="24" t="n">
         <f aca="false">Segments!G12</f>
-        <v>1799.2066934016</v>
+        <v>1632.6134810496</v>
       </c>
       <c r="E9" s="24" t="n">
         <f aca="false">Segments!H12</f>
-        <v>2101.29571846656</v>
+        <v>1979.12736274176</v>
       </c>
       <c r="F9" s="24" t="n">
         <f aca="false">Segments!I12</f>
-        <v>2335.37028803528</v>
+        <v>2203.42846385249</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5691,23 +5691,23 @@
       </c>
       <c r="B10" s="24" t="n">
         <f aca="false">B9*(1-Assumptions!$B$7)</f>
-        <v>788.7343113</v>
+        <v>417.9617718</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">C9*(1-Assumptions!$B$7)</f>
-        <v>1129.710221262</v>
+        <v>976.008150342</v>
       </c>
       <c r="D10" s="24" t="n">
         <f aca="false">D9*(1-Assumptions!$B$7)</f>
-        <v>1394.38518738624</v>
+        <v>1265.27544781344</v>
       </c>
       <c r="E10" s="24" t="n">
         <f aca="false">E9*(1-Assumptions!$B$7)</f>
-        <v>1628.50418181158</v>
+        <v>1533.82370612486</v>
       </c>
       <c r="F10" s="24" t="n">
         <f aca="false">F9*(1-Assumptions!$B$7)</f>
-        <v>1809.91197322734</v>
+        <v>1707.65705948568</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5766,19 +5766,19 @@
       </c>
       <c r="B13" s="24" t="n">
         <f aca="false">B6*Assumptions!C45</f>
-        <v>9394.35408</v>
+        <v>9742.29312</v>
       </c>
       <c r="C13" s="24" t="n">
         <f aca="false">C6*Assumptions!D45</f>
-        <v>10213.7505192</v>
+        <v>10511.2383984</v>
       </c>
       <c r="D13" s="24" t="n">
         <f aca="false">D6*Assumptions!E45</f>
-        <v>10884.089873664</v>
+        <v>11106.2141568</v>
       </c>
       <c r="E13" s="24" t="n">
         <f aca="false">E6*Assumptions!F45</f>
-        <v>11361.6570824064</v>
+        <v>11483.8254381312</v>
       </c>
       <c r="F13" s="24" t="n">
         <f aca="false">F6*Assumptions!G45</f>
@@ -5791,23 +5791,23 @@
       </c>
       <c r="B14" s="24" t="n">
         <f aca="false">-(B13-Assumptions!$B$52)</f>
-        <v>2605.64592</v>
+        <v>2897.70688</v>
       </c>
       <c r="C14" s="6" t="n">
         <f aca="false">-(C13-B13)</f>
-        <v>-819.3964392</v>
+        <v>-768.945278399999</v>
       </c>
       <c r="D14" s="6" t="n">
         <f aca="false">-(D13-C13)</f>
-        <v>-670.339354464002</v>
+        <v>-594.975758400002</v>
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">-(E13-D13)</f>
-        <v>-477.567208742401</v>
+        <v>-377.611281331201</v>
       </c>
       <c r="F14" s="6" t="n">
         <f aca="false">-(F13-E13)</f>
-        <v>-249.223445678594</v>
+        <v>-127.055089953794</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5816,23 +5816,23 @@
       </c>
       <c r="B15" s="19" t="n">
         <f aca="false">B10+B11+B12+B14</f>
-        <v>3368.2848033</v>
+        <v>3289.5732238</v>
       </c>
       <c r="C15" s="19" t="n">
         <f aca="false">C10+C11+C12+C14</f>
-        <v>280.564994142</v>
+        <v>177.314084022002</v>
       </c>
       <c r="D15" s="19" t="n">
         <f aca="false">D10+D11+D12+D14</f>
-        <v>690.727190451838</v>
+        <v>636.981046943039</v>
       </c>
       <c r="E15" s="19" t="n">
         <f aca="false">E10+E11+E12+E14</f>
-        <v>1114.28646635174</v>
+        <v>1119.56191807622</v>
       </c>
       <c r="F15" s="19" t="n">
         <f aca="false">F10+F11+F12+F14</f>
-        <v>1521.10598029391</v>
+        <v>1541.01942227705</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5841,23 +5841,23 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">Assumptions!C48</f>
-        <v>0.225730752476676</v>
+        <v>0.214188789049045</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">Assumptions!D48</f>
-        <v>0.199361760039683</v>
+        <v>0.190968667422146</v>
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">Assumptions!E48</f>
-        <v>0.178266566090088</v>
+        <v>0.173553576201971</v>
       </c>
       <c r="E16" s="9" t="n">
         <f aca="false">Assumptions!F48</f>
-        <v>0.157171372140493</v>
+        <v>0.153816472819106</v>
       </c>
       <c r="F16" s="9" t="n">
         <f aca="false">Assumptions!G48</f>
-        <v>0.141349976678297</v>
+        <v>0.138723393761621</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5866,23 +5866,23 @@
       </c>
       <c r="B17" s="28" t="n">
         <f aca="false">Assumptions!C49</f>
-        <v>0.815839855514295</v>
+        <v>0.82359515177471</v>
       </c>
       <c r="C17" s="28" t="n">
         <f aca="false">Assumptions!D49</f>
-        <v>0.6802283370176</v>
+        <v>0.691533853327463</v>
       </c>
       <c r="D17" s="28" t="n">
         <f aca="false">Assumptions!E49</f>
-        <v>0.577312771654756</v>
+        <v>0.589264834048317</v>
       </c>
       <c r="E17" s="28" t="n">
         <f aca="false">Assumptions!F49</f>
-        <v>0.498899977612532</v>
+        <v>0.510709326768904</v>
       </c>
       <c r="F17" s="28" t="n">
         <f aca="false">Assumptions!G49</f>
-        <v>0.437113933330507</v>
+        <v>0.448492873305996</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5891,23 +5891,23 @@
       </c>
       <c r="B18" s="19" t="n">
         <f aca="false">B15*B17</f>
-        <v>2747.98098725527</v>
+        <v>2709.27655852958</v>
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">C15*C17</f>
-        <v>190.848259390566</v>
+        <v>122.618691772964</v>
       </c>
       <c r="D18" s="19" t="n">
         <f aca="false">D15*D17</f>
-        <v>398.765628777053</v>
+        <v>375.350530918813</v>
       </c>
       <c r="E18" s="19" t="n">
         <f aca="false">E15*E17</f>
-        <v>555.917493116833</v>
+        <v>571.770713456811</v>
       </c>
       <c r="F18" s="19" t="n">
         <f aca="false">F15*F17</f>
-        <v>664.896618058828</v>
+        <v>691.136228517381</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5916,7 +5916,7 @@
       </c>
       <c r="B20" s="19" t="n">
         <f aca="false">SUM(B18:F18)</f>
-        <v>4558.40898659855</v>
+        <v>4470.15272319555</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5925,7 +5925,7 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">F10/(F13+0.05*F6)</f>
-        <v>0.1475</v>
+        <v>0.139166666666667</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5934,7 +5934,7 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">Assumptions!$B$26/B21</f>
-        <v>0.338983050847458</v>
+        <v>0.359281437125749</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="B23" s="6" t="n">
         <f aca="false">F10*(1+Assumptions!$B$26)*(1-B22)</f>
-        <v>1256.20161531626</v>
+        <v>1148.83395588752</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="B24" s="6" t="n">
         <f aca="false">B23/(Assumptions!$B$25-Assumptions!$B$26)</f>
-        <v>13751.5263932707</v>
+        <v>12948.4897632993</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5961,7 +5961,7 @@
       </c>
       <c r="B25" s="6" t="n">
         <f aca="false">B24*F17</f>
-        <v>6010.98379106081</v>
+        <v>5807.30537891538</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5970,7 +5970,7 @@
       </c>
       <c r="B26" s="19" t="n">
         <f aca="false">B20+B25</f>
-        <v>10569.3927776594</v>
+        <v>10277.4581021109</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">B25/B26</f>
-        <v>0.568716095381212</v>
+        <v>0.565052693109261</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="B28" s="24" t="n">
         <f aca="false">-Assumptions!$B$28</f>
-        <v>-8800</v>
+        <v>-10200</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="B30" s="19" t="n">
         <f aca="false">B26-Assumptions!$B$28-Assumptions!$B$29</f>
-        <v>1769.39277765935</v>
+        <v>77.4581021109334</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">B30/Assumptions!$B$6</f>
-        <v>0.533988597838447</v>
+        <v>0.0233762361074855</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6024,7 +6024,7 @@
       </c>
       <c r="B32" s="20" t="n">
         <f aca="false">B31/Assumptions!$B$5-1</f>
-        <v>-0.756169590028107</v>
+        <v>-0.989325919585623</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6150,23 +6150,23 @@
       </c>
       <c r="E7" s="24" t="n">
         <f aca="false">Segments!E9</f>
-        <v>1130.80188</v>
+        <v>652.3857</v>
       </c>
       <c r="F7" s="24" t="n">
         <f aca="false">Segments!F9</f>
-        <v>1586.6020224</v>
+        <v>1388.2767696</v>
       </c>
       <c r="G7" s="24" t="n">
         <f aca="false">Segments!G9</f>
-        <v>1943.58747744</v>
+        <v>1776.994265088</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">Segments!H9</f>
-        <v>2260.1145809088</v>
+        <v>2137.946225184</v>
       </c>
       <c r="I7" s="24" t="n">
         <f aca="false">Segments!I9</f>
-        <v>2506.8946594729</v>
+        <v>2374.95283529011</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6218,23 +6218,23 @@
       </c>
       <c r="E9" s="23" t="n">
         <f aca="false">Segments!E12</f>
-        <v>1017.721692</v>
+        <v>539.305512</v>
       </c>
       <c r="F9" s="23" t="n">
         <f aca="false">Segments!F12</f>
-        <v>1457.69060808</v>
+        <v>1259.36535528</v>
       </c>
       <c r="G9" s="23" t="n">
         <f aca="false">Segments!G12</f>
-        <v>1799.2066934016</v>
+        <v>1632.6134810496</v>
       </c>
       <c r="H9" s="23" t="n">
         <f aca="false">Segments!H12</f>
-        <v>2101.29571846656</v>
+        <v>1979.12736274176</v>
       </c>
       <c r="I9" s="23" t="n">
         <f aca="false">Segments!I12</f>
-        <v>2335.37028803528</v>
+        <v>2203.42846385249</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6252,23 +6252,23 @@
       </c>
       <c r="E10" s="24" t="n">
         <f aca="false">-Assumptions!C46*Assumptions!$B$28</f>
-        <v>-2068</v>
+        <v>-2244</v>
       </c>
       <c r="F10" s="24" t="n">
         <f aca="false">-Assumptions!D46*'Balance Sheet'!D11</f>
-        <v>-1526.85284136</v>
+        <v>-1806.6166072</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">-Assumptions!E46*'Balance Sheet'!E11</f>
-        <v>-1555.916702516</v>
+        <v>-1920.1202455344</v>
       </c>
       <c r="H10" s="24" t="n">
         <f aca="false">-Assumptions!F46*'Balance Sheet'!F11</f>
-        <v>-1470.3985580163</v>
+        <v>-1897.53135929199</v>
       </c>
       <c r="I10" s="24" t="n">
         <f aca="false">-Assumptions!G46*'Balance Sheet'!G11</f>
-        <v>-1322.57219480605</v>
+        <v>-1802.26177215008</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6286,23 +6286,23 @@
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">E9+E10</f>
-        <v>-1050.278308</v>
+        <v>-1704.694488</v>
       </c>
       <c r="F11" s="19" t="n">
         <f aca="false">F9+F10</f>
-        <v>-69.1622332799998</v>
+        <v>-547.25125192</v>
       </c>
       <c r="G11" s="19" t="n">
         <f aca="false">G9+G10</f>
-        <v>243.2899908856</v>
+        <v>-287.5067644848</v>
       </c>
       <c r="H11" s="19" t="n">
         <f aca="false">H9+H10</f>
-        <v>630.897160450264</v>
+        <v>81.5960034497662</v>
       </c>
       <c r="I11" s="19" t="n">
         <f aca="false">I9+I10</f>
-        <v>1012.79809322923</v>
+        <v>401.166691702412</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6311,23 +6311,23 @@
       </c>
       <c r="E12" s="6" t="n">
         <f aca="false">SUM($E$11:E11)</f>
-        <v>-1050.278308</v>
+        <v>-1704.694488</v>
       </c>
       <c r="F12" s="6" t="n">
         <f aca="false">SUM($E$11:F11)</f>
-        <v>-1119.44054128</v>
+        <v>-2251.94573992</v>
       </c>
       <c r="G12" s="6" t="n">
         <f aca="false">SUM($E$11:G11)</f>
-        <v>-876.150550394399</v>
+        <v>-2539.4525044048</v>
       </c>
       <c r="H12" s="6" t="n">
         <f aca="false">SUM($E$11:H11)</f>
-        <v>-245.253389944135</v>
+        <v>-2457.85650095503</v>
       </c>
       <c r="I12" s="6" t="n">
         <f aca="false">SUM($E$11:I11)</f>
-        <v>767.544703285094</v>
+        <v>-2056.68980925262</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6361,7 +6361,7 @@
       </c>
       <c r="I13" s="24" t="n">
         <f aca="false">-(Assumptions!$B$7*MAX(0,I12)-Assumptions!$B$7*MAX(0,F12))</f>
-        <v>-172.697558239146</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6379,23 +6379,23 @@
       </c>
       <c r="E14" s="19" t="n">
         <f aca="false">E11+E13</f>
-        <v>-1050.278308</v>
+        <v>-1704.694488</v>
       </c>
       <c r="F14" s="19" t="n">
         <f aca="false">F11+F13</f>
-        <v>-69.1622332799998</v>
+        <v>-547.25125192</v>
       </c>
       <c r="G14" s="19" t="n">
         <f aca="false">G11+G13</f>
-        <v>243.2899908856</v>
+        <v>-287.5067644848</v>
       </c>
       <c r="H14" s="19" t="n">
         <f aca="false">H11+H13</f>
-        <v>630.897160450264</v>
+        <v>81.5960034497662</v>
       </c>
       <c r="I14" s="19" t="n">
         <f aca="false">I11+I13</f>
-        <v>840.100534990083</v>
+        <v>401.166691702412</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6416,23 +6416,23 @@
       </c>
       <c r="E15" s="8" t="n">
         <f aca="false">E14/Assumptions!$B$6</f>
-        <v>-0.316965598656371</v>
+        <v>-0.514463171141811</v>
       </c>
       <c r="F15" s="8" t="n">
         <f aca="false">F14/Assumptions!$B$6</f>
-        <v>-0.0208726092017952</v>
+        <v>-0.165156053742159</v>
       </c>
       <c r="G15" s="8" t="n">
         <f aca="false">G14/Assumptions!$B$6</f>
-        <v>0.0734229746732591</v>
+        <v>-0.0867672435282562</v>
       </c>
       <c r="H15" s="8" t="n">
         <f aca="false">H14/Assumptions!$B$6</f>
-        <v>0.190399720368901</v>
+        <v>0.0246250216579951</v>
       </c>
       <c r="I15" s="8" t="n">
         <f aca="false">I14/Assumptions!$B$6</f>
-        <v>0.2535356266776</v>
+        <v>0.121068901097832</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
ELEC rev 4a: surface TV%-of-EV at summary level; make TV-share disclosure a standing protocol rule
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDB3U7m8U6NX4ju3RCn348
</commit_message>
<xml_diff>
--- a/engine/elec_study/ELEC_Valuation_Model_05082026_public.xlsx
+++ b/engine/elec_study/ELEC_Valuation_Model_05082026_public.xlsx
@@ -3417,7 +3417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3596,8 +3596,19 @@
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Terminal value share of DCF enterprise value</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>DCF!B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Read: meaningfully overvalued — the price capitalises devaluation-era earnings; the swing factors are working-capital collection, margin normalisation, and the easing path.</t>
         </is>

</xml_diff>

<commit_message>
ELEC rev 5: external-audit response — copper re-anchored to market ($14k), ownership/peers corrected, all verified prose-model inconsistencies fixed, bull bridge and terminal-ROIC grid published
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDB3U7m8U6NX4ju3RCn348
</commit_message>
<xml_diff>
--- a/engine/elec_study/ELEC_Valuation_Model_05082026_public.xlsx
+++ b/engine/elec_study/ELEC_Valuation_Model_05082026_public.xlsx
@@ -1432,7 +1432,7 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>No dividends modelled — the company has never paid one and the balance sheet argues against a first.</t>
+          <t>No dividends modelled — none in the disclosed record and the balance sheet argues against a first.</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2238,19 +2238,19 @@
         <v>0.129988</v>
       </c>
       <c r="B9" s="39" t="n">
-        <v>-0.87</v>
+        <v>-1.31</v>
       </c>
       <c r="C9" s="39" t="n">
-        <v>-0.92</v>
+        <v>-1.4</v>
       </c>
       <c r="D9" s="39" t="n">
-        <v>-0.98</v>
+        <v>-1.51</v>
       </c>
       <c r="E9" s="39" t="n">
-        <v>-1.07</v>
+        <v>-1.66</v>
       </c>
       <c r="F9" s="39" t="n">
-        <v>-1.2</v>
+        <v>-1.87</v>
       </c>
     </row>
     <row r="10">
@@ -2258,19 +2258,19 @@
         <v>0.139988</v>
       </c>
       <c r="B10" s="39" t="n">
-        <v>-1.04</v>
+        <v>-1.48</v>
       </c>
       <c r="C10" s="39" t="n">
-        <v>-1.1</v>
+        <v>-1.56</v>
       </c>
       <c r="D10" s="39" t="n">
-        <v>-1.17</v>
+        <v>-1.68</v>
       </c>
       <c r="E10" s="39" t="n">
-        <v>-1.27</v>
+        <v>-1.82</v>
       </c>
       <c r="F10" s="39" t="n">
-        <v>-1.39</v>
+        <v>-2.02</v>
       </c>
     </row>
     <row r="11">
@@ -2278,19 +2278,19 @@
         <v>0.149988</v>
       </c>
       <c r="B11" s="39" t="n">
-        <v>-1.19</v>
+        <v>-1.61</v>
       </c>
       <c r="C11" s="39" t="n">
-        <v>-1.25</v>
+        <v>-1.7</v>
       </c>
       <c r="D11" s="39" t="n">
-        <v>-1.32</v>
+        <v>-1.81</v>
       </c>
       <c r="E11" s="39" t="n">
-        <v>-1.42</v>
+        <v>-1.95</v>
       </c>
       <c r="F11" s="39" t="n">
-        <v>-1.54</v>
+        <v>-2.13</v>
       </c>
     </row>
     <row r="12">
@@ -2298,19 +2298,19 @@
         <v>0.159988</v>
       </c>
       <c r="B12" s="39" t="n">
-        <v>-1.31</v>
+        <v>-1.72</v>
       </c>
       <c r="C12" s="39" t="n">
-        <v>-1.37</v>
+        <v>-1.81</v>
       </c>
       <c r="D12" s="39" t="n">
-        <v>-1.44</v>
+        <v>-1.92</v>
       </c>
       <c r="E12" s="39" t="n">
-        <v>-1.54</v>
+        <v>-2.05</v>
       </c>
       <c r="F12" s="39" t="n">
-        <v>-1.66</v>
+        <v>-2.21</v>
       </c>
     </row>
     <row r="13">
@@ -2318,19 +2318,19 @@
         <v>0.169988</v>
       </c>
       <c r="B13" s="39" t="n">
-        <v>-1.41</v>
+        <v>-1.82</v>
       </c>
       <c r="C13" s="39" t="n">
-        <v>-1.47</v>
+        <v>-1.9</v>
       </c>
       <c r="D13" s="39" t="n">
-        <v>-1.55</v>
+        <v>-2</v>
       </c>
       <c r="E13" s="39" t="n">
-        <v>-1.64</v>
+        <v>-2.13</v>
       </c>
       <c r="F13" s="39" t="n">
-        <v>-1.75</v>
+        <v>-2.28</v>
       </c>
     </row>
     <row r="15">
@@ -2367,19 +2367,19 @@
         <v>0.1952611846539747</v>
       </c>
       <c r="B17" s="39" t="n">
-        <v>-0.91</v>
+        <v>-1.46</v>
       </c>
       <c r="C17" s="39" t="n">
-        <v>-1.11</v>
+        <v>-1.63</v>
       </c>
       <c r="D17" s="39" t="n">
-        <v>-1.27</v>
+        <v>-1.77</v>
       </c>
       <c r="E17" s="39" t="n">
-        <v>-1.39</v>
+        <v>-1.88</v>
       </c>
       <c r="F17" s="39" t="n">
-        <v>-1.5</v>
+        <v>-1.97</v>
       </c>
     </row>
     <row r="18">
@@ -2387,19 +2387,19 @@
         <v>0.2052611846539747</v>
       </c>
       <c r="B18" s="39" t="n">
-        <v>-0.95</v>
+        <v>-1.49</v>
       </c>
       <c r="C18" s="39" t="n">
-        <v>-1.14</v>
+        <v>-1.65</v>
       </c>
       <c r="D18" s="39" t="n">
-        <v>-1.29</v>
+        <v>-1.79</v>
       </c>
       <c r="E18" s="39" t="n">
-        <v>-1.42</v>
+        <v>-1.9</v>
       </c>
       <c r="F18" s="39" t="n">
-        <v>-1.52</v>
+        <v>-1.99</v>
       </c>
     </row>
     <row r="19">
@@ -2407,19 +2407,19 @@
         <v>0.2152611846539747</v>
       </c>
       <c r="B19" s="39" t="n">
-        <v>-0.98</v>
+        <v>-1.51</v>
       </c>
       <c r="C19" s="39" t="n">
-        <v>-1.17</v>
+        <v>-1.68</v>
       </c>
       <c r="D19" s="39" t="n">
-        <v>-1.32</v>
+        <v>-1.81</v>
       </c>
       <c r="E19" s="39" t="n">
-        <v>-1.44</v>
+        <v>-1.92</v>
       </c>
       <c r="F19" s="39" t="n">
-        <v>-1.55</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="20">
@@ -2427,19 +2427,19 @@
         <v>0.2252611846539747</v>
       </c>
       <c r="B20" s="39" t="n">
-        <v>-1.02</v>
+        <v>-1.54</v>
       </c>
       <c r="C20" s="39" t="n">
-        <v>-1.2</v>
+        <v>-1.7</v>
       </c>
       <c r="D20" s="39" t="n">
-        <v>-1.35</v>
+        <v>-1.83</v>
       </c>
       <c r="E20" s="39" t="n">
-        <v>-1.47</v>
+        <v>-1.93</v>
       </c>
       <c r="F20" s="39" t="n">
-        <v>-1.57</v>
+        <v>-2.02</v>
       </c>
     </row>
     <row r="21">
@@ -2447,19 +2447,19 @@
         <v>0.2352611846539747</v>
       </c>
       <c r="B21" s="39" t="n">
-        <v>-1.05</v>
+        <v>-1.56</v>
       </c>
       <c r="C21" s="39" t="n">
-        <v>-1.23</v>
+        <v>-1.72</v>
       </c>
       <c r="D21" s="39" t="n">
-        <v>-1.37</v>
+        <v>-1.85</v>
       </c>
       <c r="E21" s="39" t="n">
-        <v>-1.49</v>
+        <v>-1.95</v>
       </c>
       <c r="F21" s="39" t="n">
-        <v>-1.59</v>
+        <v>-2.04</v>
       </c>
     </row>
     <row r="23">
@@ -2496,19 +2496,19 @@
         <v>-0.3</v>
       </c>
       <c r="B25" s="39" t="n">
-        <v>-2.72</v>
+        <v>-3.26</v>
       </c>
       <c r="C25" s="39" t="n">
-        <v>-2.5</v>
+        <v>-3.02</v>
       </c>
       <c r="D25" s="39" t="n">
+        <v>-2.77</v>
+      </c>
+      <c r="E25" s="39" t="n">
+        <v>-2.53</v>
+      </c>
+      <c r="F25" s="39" t="n">
         <v>-2.29</v>
-      </c>
-      <c r="E25" s="39" t="n">
-        <v>-2.07</v>
-      </c>
-      <c r="F25" s="39" t="n">
-        <v>-1.85</v>
       </c>
     </row>
     <row r="26">
@@ -2516,19 +2516,19 @@
         <v>-0.15</v>
       </c>
       <c r="B26" s="39" t="n">
-        <v>-2.24</v>
+        <v>-2.77</v>
       </c>
       <c r="C26" s="39" t="n">
-        <v>-2.02</v>
+        <v>-2.53</v>
       </c>
       <c r="D26" s="39" t="n">
-        <v>-1.8</v>
+        <v>-2.29</v>
       </c>
       <c r="E26" s="39" t="n">
-        <v>-1.59</v>
+        <v>-2.05</v>
       </c>
       <c r="F26" s="39" t="n">
-        <v>-1.37</v>
+        <v>-1.81</v>
       </c>
     </row>
     <row r="27">
@@ -2536,19 +2536,19 @@
         <v>0</v>
       </c>
       <c r="B27" s="39" t="n">
-        <v>-1.76</v>
+        <v>-2.29</v>
       </c>
       <c r="C27" s="39" t="n">
-        <v>-1.54</v>
+        <v>-2.05</v>
       </c>
       <c r="D27" s="39" t="n">
-        <v>-1.32</v>
+        <v>-1.81</v>
       </c>
       <c r="E27" s="39" t="n">
-        <v>-1.1</v>
+        <v>-1.57</v>
       </c>
       <c r="F27" s="39" t="n">
-        <v>-0.89</v>
+        <v>-1.33</v>
       </c>
     </row>
     <row r="28">
@@ -2556,19 +2556,19 @@
         <v>0.15</v>
       </c>
       <c r="B28" s="39" t="n">
-        <v>-1.27</v>
+        <v>-1.81</v>
       </c>
       <c r="C28" s="39" t="n">
-        <v>-1.06</v>
+        <v>-1.57</v>
       </c>
       <c r="D28" s="39" t="n">
+        <v>-1.33</v>
+      </c>
+      <c r="E28" s="39" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="F28" s="39" t="n">
         <v>-0.84</v>
-      </c>
-      <c r="E28" s="39" t="n">
-        <v>-0.62</v>
-      </c>
-      <c r="F28" s="39" t="n">
-        <v>-0.4</v>
       </c>
     </row>
     <row r="29">
@@ -2576,172 +2576,281 @@
         <v>0.3</v>
       </c>
       <c r="B29" s="39" t="n">
-        <v>-0.79</v>
+        <v>-1.33</v>
       </c>
       <c r="C29" s="39" t="n">
-        <v>-0.57</v>
+        <v>-1.08</v>
       </c>
       <c r="D29" s="39" t="n">
-        <v>-0.35</v>
+        <v>-0.84</v>
       </c>
       <c r="E29" s="39" t="n">
-        <v>-0.14</v>
+        <v>-0.6</v>
       </c>
       <c r="F29" s="39" t="n">
-        <v>0.08</v>
+        <v>-0.36</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Beta grid (Ke / WACCs / DCF)</t>
+          <t>Terminal-ROIC grid (drives RR = g/ROIC and the inverted g-gradient)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
+          <t>Terminal ROIC</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>RR for g=5%</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Terminal value</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>DCF (EGP/sh, unfloored)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>0.077</v>
+      </c>
+      <c r="B33" s="12" t="n">
+        <v>0.6493506493506493</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>5513</v>
+      </c>
+      <c r="D33" s="39" t="n">
+        <v>-2.02</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="B34" s="12" t="n">
+        <v>0.5882352941176471</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>6474</v>
+      </c>
+      <c r="D34" s="39" t="n">
+        <v>-1.9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>0.09170814583433977</v>
+      </c>
+      <c r="B35" s="12" t="n">
+        <v>0.5452078389014566</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>7150</v>
+      </c>
+      <c r="D35" s="39" t="n">
+        <v>-1.81</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="B36" s="12" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>9171</v>
+      </c>
+      <c r="D36" s="39" t="n">
+        <v>-1.54</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B37" s="12" t="n">
+        <v>0.3333333333333334</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>10481</v>
+      </c>
+      <c r="D37" s="39" t="n">
+        <v>-1.37</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Challenged net-debt reading (unverified aggregator 10,386): DCF unfloored</t>
+        </is>
+      </c>
+      <c r="E39" s="39" t="n">
+        <v>-1.98</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Beta grid (Ke / WACCs / DCF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>Ke</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>WACC explicit</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>WACC terminal</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>DCF (EGP/sh)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="39" t="n">
+    <row r="43">
+      <c r="A43" s="39" t="n">
         <v>0.6</v>
       </c>
-      <c r="B33" s="12" t="n">
+      <c r="B43" s="12" t="n">
         <v>0.24556</v>
       </c>
-      <c r="C33" s="12" t="n">
+      <c r="C43" s="12" t="n">
         <v>0.2012355297306375</v>
       </c>
-      <c r="D33" s="12" t="n">
+      <c r="D43" s="12" t="n">
         <v>0.1347</v>
       </c>
-      <c r="E33" s="39" t="n">
-        <v>-1.08</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="39" t="n">
+      <c r="E43" s="39" t="n">
+        <v>-1.59</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="39" t="n">
         <v>0.78</v>
       </c>
-      <c r="B34" s="12" t="n">
+      <c r="B44" s="12" t="n">
         <v>0.262498</v>
       </c>
-      <c r="C34" s="12" t="n">
+      <c r="C44" s="12" t="n">
         <v>0.2081712931542658</v>
       </c>
-      <c r="D34" s="12" t="n">
+      <c r="D44" s="12" t="n">
         <v>0.14226</v>
       </c>
-      <c r="E34" s="39" t="n">
-        <v>-1.21</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="39" t="n">
+      <c r="E44" s="39" t="n">
+        <v>-1.71</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="39" t="n">
         <v>0.8</v>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B45" s="12" t="n">
         <v>0.26438</v>
       </c>
-      <c r="C35" s="12" t="n">
+      <c r="C45" s="12" t="n">
         <v>0.2089419335346689</v>
       </c>
-      <c r="D35" s="12" t="n">
+      <c r="D45" s="12" t="n">
         <v>0.1431</v>
       </c>
-      <c r="E35" s="39" t="n">
-        <v>-1.22</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="39" t="n">
+      <c r="E45" s="39" t="n">
+        <v>-1.72</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="39" t="n">
         <v>0.964</v>
       </c>
-      <c r="B36" s="12" t="n">
+      <c r="B46" s="12" t="n">
         <v>0.2798124</v>
       </c>
-      <c r="C36" s="12" t="n">
+      <c r="C46" s="12" t="n">
         <v>0.2152611846539747</v>
       </c>
-      <c r="D36" s="12" t="n">
+      <c r="D46" s="12" t="n">
         <v>0.149988</v>
       </c>
-      <c r="E36" s="39" t="n">
-        <v>-1.32</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="39" t="n">
+      <c r="E46" s="39" t="n">
+        <v>-1.81</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="B37" s="12" t="n">
+      <c r="B47" s="12" t="n">
         <v>0.2832</v>
       </c>
-      <c r="C37" s="12" t="n">
+      <c r="C47" s="12" t="n">
         <v>0.2166483373387004</v>
       </c>
-      <c r="D37" s="12" t="n">
+      <c r="D47" s="12" t="n">
         <v>0.1515</v>
       </c>
-      <c r="E37" s="39" t="n">
-        <v>-1.34</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="39" t="n">
+      <c r="E47" s="39" t="n">
+        <v>-1.83</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="39" t="n">
         <v>1.15</v>
       </c>
-      <c r="B38" s="12" t="n">
+      <c r="B48" s="12" t="n">
         <v>0.297315</v>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C48" s="12" t="n">
         <v>0.222428140191724</v>
       </c>
-      <c r="D38" s="12" t="n">
+      <c r="D48" s="12" t="n">
         <v>0.1578</v>
       </c>
-      <c r="E38" s="39" t="n">
-        <v>-1.42</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="39" t="n">
+      <c r="E48" s="39" t="n">
+        <v>-1.89</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="39" t="n">
         <v>1.3</v>
       </c>
-      <c r="B39" s="12" t="n">
+      <c r="B49" s="12" t="n">
         <v>0.31143</v>
       </c>
-      <c r="C39" s="12" t="n">
+      <c r="C49" s="12" t="n">
         <v>0.2282079430447475</v>
       </c>
-      <c r="D39" s="12" t="n">
+      <c r="D49" s="12" t="n">
         <v>0.1641</v>
       </c>
-      <c r="E39" s="39" t="n">
-        <v>-1.49</v>
+      <c r="E49" s="39" t="n">
+        <v>-1.95</v>
       </c>
     </row>
   </sheetData>
@@ -3272,17 +3381,17 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>EGP 196bn</t>
+          <t>EGP 196bn (21-Jul; ~205bn 27-Jul)</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>10.4x</t>
+          <t>11.3x computed</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>~6.0x</t>
+          <t>~7.1x computed</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
@@ -3292,7 +3401,7 @@
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>FY25 rev EGP 281bn, NP 17.3bn; W&amp;C segment +66% — the demand proof</t>
+          <t>FY25 rev 281bn, NP 17.3bn, EBITDA 30.7bn, net bank debt 19.8bn (filed); W&amp;C grew low-teens FY25 (+66% is FY2024)</t>
         </is>
       </c>
     </row>
@@ -3304,27 +3413,27 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>SAR 18.0bn</t>
+          <t>SAR 15.4bn (30-Jul)</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>18.0x</t>
+          <t>14.3x</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>15.0x</t>
+          <t>~12.5x derived</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>0.27x</t>
+          <t>~0.5x</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Same industry, clean balance sheet, different market</t>
+          <t>Same industry, clean balance sheet, different market; BS inputs unverified</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3594,7 @@
         <v/>
       </c>
       <c r="D6" s="7" t="n">
-        <v>1.54</v>
+        <v>1.01</v>
       </c>
       <c r="E6" s="9">
         <f>Assumptions!B35</f>
@@ -3520,14 +3629,14 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="C8" s="8">
         <f>'Relative &amp; Normalized'!C7</f>
         <v/>
       </c>
       <c r="D8" s="7" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="E8" s="9">
         <f>Assumptions!B37</f>
@@ -3548,7 +3657,7 @@
         <v/>
       </c>
       <c r="D9" s="7" t="n">
-        <v>1.43</v>
+        <v>1.31</v>
       </c>
       <c r="E9" s="9">
         <f>Assumptions!B38</f>
@@ -4184,7 +4293,7 @@
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>SWDY ~6.0x; discount for leverage/concentration</t>
+          <t>SWDY ~7.1x COMPUTED from its FY25 filing (prior 6.0x aggregator print did not reproduce); discount for leverage/concentration</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4308,7 @@
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>SWDY 10.4x trailing; deep discount</t>
+          <t>SWDY 11.3x COMPUTED (prior 10.4x did not reproduce); ~42% discount held deliberately deep</t>
         </is>
       </c>
     </row>
@@ -4346,23 +4455,23 @@
         </is>
       </c>
       <c r="C42" s="23" t="n">
-        <v>12600</v>
+        <v>14000</v>
       </c>
       <c r="D42" s="23" t="n">
-        <v>12600</v>
+        <v>14000</v>
       </c>
       <c r="E42" s="23" t="n">
-        <v>12600</v>
+        <v>14000</v>
       </c>
       <c r="F42" s="23" t="n">
-        <v>12600</v>
+        <v>14000</v>
       </c>
       <c r="G42" s="23" t="n">
-        <v>12600</v>
+        <v>14000</v>
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
-          <t>Flat at the 2026 consensus avg — no house commodity view; bull/bear move it</t>
+          <t>Flat at the CURRENT market (~$14.0k LME cash 3-4 Aug-26); the -10% sensitivity (=12.6k) is the mean-reversion case</t>
         </is>
       </c>
     </row>

</xml_diff>